<commit_message>
progress: 62 village workbooks (sivaramans-llin 2026-10-10T16:00:00Z)
</commit_message>
<xml_diff>
--- a/out/Village_map_of_Tiruvallur_Gummidipoondi_Peruvoyal_13.343408_80.14676.xlsx
+++ b/out/Village_map_of_Tiruvallur_Gummidipoondi_Peruvoyal_13.343408_80.14676.xlsx
@@ -1070,6 +1070,11 @@
           <t>153</t>
         </is>
       </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 2C1, 2C2, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -1077,6 +1082,11 @@
           <t>154</t>
         </is>
       </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>1, 2A1A1, 2A1A2, 2A1B, 2A2, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -1084,6 +1094,11 @@
           <t>155</t>
         </is>
       </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>10, 11, 12, 1A1, 1A2, 1B1, 1B2, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -1091,6 +1106,11 @@
           <t>156</t>
         </is>
       </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6, 7, 8A, 8B, 8C, 8D, 9</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -1098,6 +1118,11 @@
           <t>157</t>
         </is>
       </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>2, 3, 4, 5, 6A1, 6A2, 6B, 7</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -1105,6 +1130,11 @@
           <t>158</t>
         </is>
       </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13A, 13B, 2, 3, 4, 5, 6, 7, 8, 9A, 9B</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -1112,6 +1142,11 @@
           <t>159</t>
         </is>
       </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 2, 3A, 3B, 4A, 4B, 5A, 5B, 6A, 6B, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -1119,6 +1154,11 @@
           <t>160</t>
         </is>
       </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 1D, 2A, 2B, 3, 4A, 4B</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -1126,6 +1166,11 @@
           <t>161</t>
         </is>
       </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>10A, 10B, 11A, 11B, 12A, 12B, 13, 14A1, 14A2, 14B1A, 14B1B, 14B2, 1A, 1B, 1C, 2A, 2B, 3, 4, 5A, 5B, 5C, 5D, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -1133,6 +1178,11 @@
           <t>162</t>
         </is>
       </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -1140,6 +1190,11 @@
           <t>163</t>
         </is>
       </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -1147,6 +1202,11 @@
           <t>164</t>
         </is>
       </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>1A, 1A1A, 1A1B, 1A2, 1A3, 1B1A, 1B1B, 1B2, 2, 2A1, 2A2, 2B, 3, 4A, 4C1A1, 4C1A2, 4C1B, 4C2A1, 4C2A2, 4C2A3, 4C2B, 4C2C, 5A, 5A1A, 5A1B, 5A2, 5B1, 5B2, 8, 8A, 8B, 8C</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -1154,6 +1214,11 @@
           <t>165</t>
         </is>
       </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>10, 10A1, 10A2, 10C, 11A1, 11A2A, 11A2B, 11B, 1A1, 1A2, 1B, 2, 3, 4, 5, 6, 7, 8, 9A, 9B, 9C</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -1161,6 +1226,11 @@
           <t>166</t>
         </is>
       </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -1168,6 +1238,11 @@
           <t>167</t>
         </is>
       </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -1175,6 +1250,11 @@
           <t>168</t>
         </is>
       </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -1182,6 +1262,11 @@
           <t>169</t>
         </is>
       </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -1189,6 +1274,11 @@
           <t>170</t>
         </is>
       </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -1196,6 +1286,11 @@
           <t>171</t>
         </is>
       </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>1, 2, 3A1, 3A2, 3B, 4, 5, 6, 7, 8</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -1203,6 +1298,11 @@
           <t>172</t>
         </is>
       </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -1210,6 +1310,11 @@
           <t>173</t>
         </is>
       </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3A1, 3A2, 3B, 4, 5A1, 5A2, 5B1, 5B2, 5C, 6</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -1217,6 +1322,11 @@
           <t>174</t>
         </is>
       </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>1A, 1B1A, 1B1B, 1B2A1, 1B2A2, 1B2B, 2, 3, 4, 5, 6, 7A, 7B, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -1224,6 +1334,11 @@
           <t>175</t>
         </is>
       </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>1, 10, 11A, 11B, 12, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -1231,6 +1346,11 @@
           <t>176</t>
         </is>
       </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 2C, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -1238,6 +1358,11 @@
           <t>177</t>
         </is>
       </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6, 7</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -1245,6 +1370,11 @@
           <t>178</t>
         </is>
       </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -1252,6 +1382,11 @@
           <t>179</t>
         </is>
       </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 2, 3, 4, 5, 6, 7, 8, 9A, 9B</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -1259,6 +1394,11 @@
           <t>180</t>
         </is>
       </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>1, 2, 3A, 3B, 3C, 3D, 3E, 4</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -1266,6 +1406,11 @@
           <t>181</t>
         </is>
       </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3, 4A, 4B, 5</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -1273,6 +1418,11 @@
           <t>182</t>
         </is>
       </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -1280,6 +1430,11 @@
           <t>183</t>
         </is>
       </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -1287,6 +1442,11 @@
           <t>184</t>
         </is>
       </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -1294,6 +1454,11 @@
           <t>185</t>
         </is>
       </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -1301,6 +1466,11 @@
           <t>186</t>
         </is>
       </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B, 3A, 3B, 3C, 4</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -1308,6 +1478,11 @@
           <t>187</t>
         </is>
       </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3, 4, 5A, 5B, 6</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -1315,6 +1490,11 @@
           <t>188</t>
         </is>
       </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B, 2C, 2D, 3, 4, 5</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -1322,6 +1502,11 @@
           <t>189</t>
         </is>
       </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -1329,6 +1514,11 @@
           <t>190</t>
         </is>
       </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3, 4, 5</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -1336,6 +1526,11 @@
           <t>191</t>
         </is>
       </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -1343,6 +1538,11 @@
           <t>192</t>
         </is>
       </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>1, 2, 3A, 3B1, 3B2, 4</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -1350,6 +1550,11 @@
           <t>193</t>
         </is>
       </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -1357,6 +1562,11 @@
           <t>194</t>
         </is>
       </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>10, 11, 12, 13A, 13B, 1A1, 1A2, 1B, 2, 3, 4, 5, 6, 7, 8A, 8B, 9</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -1364,6 +1574,11 @@
           <t>195</t>
         </is>
       </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -1371,6 +1586,11 @@
           <t>196</t>
         </is>
       </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6, 7, 8</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -1378,6 +1598,11 @@
           <t>197</t>
         </is>
       </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6, 7</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -1385,6 +1610,11 @@
           <t>198</t>
         </is>
       </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1B, 2A, 2B, 2C, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -1392,6 +1622,11 @@
           <t>199</t>
         </is>
       </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6, 7, 8</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -1399,6 +1634,11 @@
           <t>200</t>
         </is>
       </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 2, 3, 4, 5, 6, 7A, 7B, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -1406,6 +1646,11 @@
           <t>201</t>
         </is>
       </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>1, 10, 2, 3A1, 3A2, 3B, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -1413,6 +1658,11 @@
           <t>202</t>
         </is>
       </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13A1, 13A2, 13A3, 13A4, 13A5, 13B, 13C, 13D, 14, 15, 16A, 16B, 16C, 17, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -1420,6 +1670,11 @@
           <t>203</t>
         </is>
       </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>10, 11, 12A, 12B, 13A, 13B, 14A, 14B, 14C, 1A, 1B, 2A, 2B, 3, 4, 5A, 5B, 6, 7A, 7B, 8, 9A, 9B</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -1427,6 +1682,11 @@
           <t>204</t>
         </is>
       </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 2A, 2B, 2C, 2D, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -1434,6 +1694,11 @@
           <t>205</t>
         </is>
       </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6A, 6B, 6C, 7A, 7B, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -1441,6 +1706,11 @@
           <t>206</t>
         </is>
       </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4A, 4B, 4C, 5A, 5B, 6A, 6B, 6C, 7, 8</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -1448,6 +1718,11 @@
           <t>207</t>
         </is>
       </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6, 7</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -1455,6 +1730,11 @@
           <t>208</t>
         </is>
       </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4A, 4B</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -1462,6 +1742,11 @@
           <t>209</t>
         </is>
       </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>1, 2, 3A, 3B, 4, 5, 6</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -1469,6 +1754,11 @@
           <t>210</t>
         </is>
       </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 2C, 2D, 2E, 2F, 2G, 2H, 2I1, 2I2, 2J, 3</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -1476,6 +1766,11 @@
           <t>211</t>
         </is>
       </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -1483,6 +1778,11 @@
           <t>212</t>
         </is>
       </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>1A1A, 1A2, 1B1, 1B2, 1C, 2A, 2B1A1A, 2B1A1B, 2B1A2, 2B1A3, 2B1A4, 2B1A5, 2B1B, 2B2A, 2B2B, 3A, 3B1, 4A1, 4A2, 4A3, 4A4A, 4A4B, 4A5, 4B, 4C, 5, 6</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -1490,6 +1790,11 @@
           <t>213</t>
         </is>
       </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -1497,6 +1802,11 @@
           <t>214</t>
         </is>
       </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 3</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -1504,6 +1814,11 @@
           <t>215</t>
         </is>
       </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3, 4, 5</t>
+        </is>
+      </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -1511,6 +1826,11 @@
           <t>216</t>
         </is>
       </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4A, 4B, 5</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -1518,6 +1838,11 @@
           <t>217</t>
         </is>
       </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -1525,6 +1850,11 @@
           <t>218</t>
         </is>
       </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 2A, 2B, 3, 4, 5, 6, 7A, 7B, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -1532,6 +1862,11 @@
           <t>219</t>
         </is>
       </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>1, 2A1A, 2A1B, 2A2A, 2A2B, 2B, 3, 4, 5A, 5B, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -1539,6 +1874,11 @@
           <t>220</t>
         </is>
       </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
@@ -1546,6 +1886,11 @@
           <t>221</t>
         </is>
       </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
@@ -1553,6 +1898,11 @@
           <t>222</t>
         </is>
       </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3, 4, 5A, 5B, 6A, 6B, 7A1, 7A2, 7B1, 7B2, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
@@ -1560,6 +1910,11 @@
           <t>223</t>
         </is>
       </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 3, 4A1, 4A2, 4A3, 4B, 5A, 5B</t>
+        </is>
+      </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
@@ -1567,6 +1922,11 @@
           <t>224</t>
         </is>
       </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
@@ -1574,6 +1934,11 @@
           <t>225</t>
         </is>
       </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
@@ -1581,6 +1946,11 @@
           <t>226</t>
         </is>
       </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>10, 11, 12, 13, 14, 15, 16, 17A, 17B, 1A, 1B, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
@@ -1588,6 +1958,11 @@
           <t>227</t>
         </is>
       </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 16, 17, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
@@ -1595,6 +1970,11 @@
           <t>228</t>
         </is>
       </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>10A, 10B, 11, 12, 1A, 1B, 2A, 2B, 3, 4, 5, 6A, 6B, 6C, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
@@ -1602,6 +1982,11 @@
           <t>229</t>
         </is>
       </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>1A, 1B1, 1B2, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
@@ -1609,6 +1994,11 @@
           <t>230</t>
         </is>
       </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>1, 10, 11A1A, 11A1B, 11A2, 11B, 2, 3, 4, 5, 6, 7A1, 7A2, 7B, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
@@ -1616,6 +2006,11 @@
           <t>231</t>
         </is>
       </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
@@ -1623,6 +2018,11 @@
           <t>232</t>
         </is>
       </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
@@ -1630,6 +2030,11 @@
           <t>233</t>
         </is>
       </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
@@ -1637,6 +2042,11 @@
           <t>234</t>
         </is>
       </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
@@ -1644,6 +2054,11 @@
           <t>235</t>
         </is>
       </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
@@ -1651,6 +2066,11 @@
           <t>236</t>
         </is>
       </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
@@ -1658,6 +2078,11 @@
           <t>237</t>
         </is>
       </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3, 4, 5</t>
+        </is>
+      </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
@@ -1665,6 +2090,11 @@
           <t>238</t>
         </is>
       </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
@@ -1672,6 +2102,11 @@
           <t>36</t>
         </is>
       </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
@@ -1679,11 +2114,21 @@
           <t>37</t>
         </is>
       </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
           <t>38</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5A, 5B, 6, 7, 8</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
progress: 63 village workbooks (sivaramans-llin 2026-10-10T16:10:00Z)
</commit_message>
<xml_diff>
--- a/out/Village_map_of_Tiruvallur_Gummidipoondi_Peruvoyal_13.343408_80.14676.xlsx
+++ b/out/Village_map_of_Tiruvallur_Gummidipoondi_Peruvoyal_13.343408_80.14676.xlsx
@@ -2138,6 +2138,11 @@
           <t>39</t>
         </is>
       </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6</t>
+        </is>
+      </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
@@ -2145,6 +2150,11 @@
           <t>40</t>
         </is>
       </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>1, 10, 2, 3, 4A, 4B, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
@@ -2152,6 +2162,11 @@
           <t>41</t>
         </is>
       </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>1, 10, 11A, 11B, 2, 3, 4, 5, 6, 7A, 7B, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
@@ -2159,6 +2174,11 @@
           <t>42</t>
         </is>
       </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6, 7, 8</t>
+        </is>
+      </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
@@ -2166,6 +2186,11 @@
           <t>43</t>
         </is>
       </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
@@ -2173,6 +2198,11 @@
           <t>44</t>
         </is>
       </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 1D, 2A, 2B, 2C, 2D, 2E, 2F, 2G, 3, 4, 5A, 5B, 6A, 6B, 7</t>
+        </is>
+      </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
@@ -2180,6 +2210,11 @@
           <t>45</t>
         </is>
       </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4A, 4B, 4C1, 4C2, 5, 6, 7</t>
+        </is>
+      </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
@@ -2187,6 +2222,11 @@
           <t>46</t>
         </is>
       </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 2, 3A, 3B, 3C, 4, 5, 6A, 6B, 6C, 6D, 6E, 6F, 7A, 7B, 8A, 8B, 8C, 9A, 9B</t>
+        </is>
+      </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
@@ -2194,6 +2234,11 @@
           <t>47</t>
         </is>
       </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12A, 12B, 12C, 13, 14, 15, 16, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
@@ -2201,6 +2246,11 @@
           <t>48</t>
         </is>
       </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>1A, 1B1, 1B2, 2</t>
+        </is>
+      </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
@@ -2208,6 +2258,11 @@
           <t>49</t>
         </is>
       </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6, 7</t>
+        </is>
+      </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
@@ -2215,6 +2270,11 @@
           <t>50</t>
         </is>
       </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>1, 2, 3A, 3B, 4A, 4B, 5</t>
+        </is>
+      </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
@@ -2222,6 +2282,11 @@
           <t>51</t>
         </is>
       </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
@@ -2229,6 +2294,11 @@
           <t>52</t>
         </is>
       </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12A, 12B, 13, 14, 15, 16, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
@@ -2236,6 +2306,11 @@
           <t>53</t>
         </is>
       </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B, 2C, 2D</t>
+        </is>
+      </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
@@ -2243,6 +2318,11 @@
           <t>54</t>
         </is>
       </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 2, 3, 4A, 4B, 4C</t>
+        </is>
+      </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
@@ -2250,6 +2330,11 @@
           <t>55</t>
         </is>
       </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6A, 6B, 6C</t>
+        </is>
+      </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
@@ -2257,6 +2342,11 @@
           <t>56</t>
         </is>
       </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1B, 1C, 2, 3, 4, 5, 6, 7</t>
+        </is>
+      </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
@@ -2264,6 +2354,11 @@
           <t>57</t>
         </is>
       </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>1, 2A1, 2A2, 2A3, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
@@ -2271,6 +2366,11 @@
           <t>58</t>
         </is>
       </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 2, 3, 4A, 4B, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
@@ -2278,6 +2378,11 @@
           <t>59</t>
         </is>
       </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>10, 11, 12, 13, 14, 1A, 1B, 1C, 2A, 2B, 3, 4, 5, 6, 7A, 7B, 7C, 7D, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
@@ -2285,6 +2390,11 @@
           <t>60</t>
         </is>
       </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6, 7, 8A, 8B, 8C, 9</t>
+        </is>
+      </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
@@ -2292,6 +2402,11 @@
           <t>61</t>
         </is>
       </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 16, 17, 2, 3A, 3B, 4, 5, 6A, 6B, 7A, 7B, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
@@ -2299,6 +2414,11 @@
           <t>62</t>
         </is>
       </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
@@ -2306,6 +2426,11 @@
           <t>63</t>
         </is>
       </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
@@ -2313,6 +2438,11 @@
           <t>64</t>
         </is>
       </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 2, 20A, 20B, 21, 3A, 3B, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
@@ -2320,6 +2450,11 @@
           <t>65</t>
         </is>
       </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
@@ -2327,6 +2462,11 @@
           <t>66</t>
         </is>
       </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
@@ -2334,6 +2474,11 @@
           <t>67</t>
         </is>
       </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>1, 10A, 10B, 11, 12, 13A, 13B, 13C, 14, 15, 16, 17, 18, 19, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
@@ -2341,6 +2486,11 @@
           <t>68</t>
         </is>
       </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
@@ -2348,6 +2498,11 @@
           <t>69</t>
         </is>
       </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
@@ -2355,6 +2510,11 @@
           <t>70</t>
         </is>
       </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 2, 3A, 3B, 4, 5, 6, 7, 8A, 8B, 8C, 8D, 9</t>
+        </is>
+      </c>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
@@ -2362,6 +2522,11 @@
           <t>71</t>
         </is>
       </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>1, 2, 3A, 3B, 4, 5, 6A, 6B, 6C, 7, 8</t>
+        </is>
+      </c>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
@@ -2369,6 +2534,11 @@
           <t>72</t>
         </is>
       </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
@@ -2376,6 +2546,11 @@
           <t>73</t>
         </is>
       </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12A, 12B, 13, 14A, 14B, 15, 16, 17, 18, 19, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
@@ -2383,6 +2558,11 @@
           <t>74</t>
         </is>
       </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 16, 17, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
@@ -2390,6 +2570,11 @@
           <t>75</t>
         </is>
       </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>1, 10, 11A, 11B, 12, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
@@ -2397,6 +2582,11 @@
           <t>76</t>
         </is>
       </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>1, 10A, 10B, 11A, 11B, 2, 3A, 3B, 4, 5A1, 5A2, 5B, 6, 7, 8A, 8B, 9A, 9B</t>
+        </is>
+      </c>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
@@ -2404,6 +2594,11 @@
           <t>77</t>
         </is>
       </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>1, 10, 11A, 11B, 12, 13, 14, 15, 16, 17, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
@@ -2411,6 +2606,11 @@
           <t>78</t>
         </is>
       </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 16, 17, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
@@ -2418,6 +2618,11 @@
           <t>79</t>
         </is>
       </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>10, 11, 12A, 12B, 13A, 13B, 14A, 14B, 1A, 1B, 2A, 2B, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
@@ -2425,6 +2630,11 @@
           <t>80</t>
         </is>
       </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 2, 3A, 3B, 4, 5, 6, 7, 8A, 8B, 9</t>
+        </is>
+      </c>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
@@ -2432,6 +2642,11 @@
           <t>81</t>
         </is>
       </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 16A, 16B, 17, 18, 2A, 2B, 2C, 2D, 3, 4A, 4B, 4C, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
@@ -2439,6 +2654,11 @@
           <t>82</t>
         </is>
       </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6, 7</t>
+        </is>
+      </c>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
@@ -2446,6 +2666,11 @@
           <t>83</t>
         </is>
       </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
@@ -2453,6 +2678,11 @@
           <t>84</t>
         </is>
       </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
@@ -2460,6 +2690,11 @@
           <t>85</t>
         </is>
       </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
@@ -2467,6 +2702,11 @@
           <t>86</t>
         </is>
       </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6</t>
+        </is>
+      </c>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
@@ -2474,6 +2714,11 @@
           <t>87</t>
         </is>
       </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
@@ -2481,6 +2726,11 @@
           <t>88</t>
         </is>
       </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>1, 2, 3A, 3B, 3C</t>
+        </is>
+      </c>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
@@ -2488,6 +2738,11 @@
           <t>89</t>
         </is>
       </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6, 7</t>
+        </is>
+      </c>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
@@ -2495,6 +2750,11 @@
           <t>90</t>
         </is>
       </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
@@ -2502,6 +2762,11 @@
           <t>91</t>
         </is>
       </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 16, 17, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
@@ -2509,6 +2774,11 @@
           <t>92</t>
         </is>
       </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>1, 2A1, 2A2, 2B, 2C, 2D, 3A1A, 3A1B, 3A2A, 3A2B, 3B1, 3B2, 4A, 4B, 5</t>
+        </is>
+      </c>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
@@ -2516,6 +2786,11 @@
           <t>93</t>
         </is>
       </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6A1, 6A2, 6B, 7A1, 7A2, 7B, 8</t>
+        </is>
+      </c>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
@@ -2523,6 +2798,11 @@
           <t>94</t>
         </is>
       </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
@@ -2530,6 +2810,11 @@
           <t>95</t>
         </is>
       </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>10, 11, 1A, 1B, 1C, 2A, 2B, 2C, 3A, 3B, 3C, 4A, 4B, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
@@ -2537,6 +2822,11 @@
           <t>96</t>
         </is>
       </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>1, 10, 11A, 11B, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
@@ -2544,6 +2834,11 @@
           <t>97</t>
         </is>
       </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
@@ -2551,11 +2846,21 @@
           <t>98</t>
         </is>
       </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
           <t>99</t>
+        </is>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>1, 10, 11A, 11B, 12, 13, 14, 15A, 15B, 15C, 16, 17A, 17B, 18, 19, 2, 20, 21, 22, 3, 4, 5, 6, 7, 8, 9</t>
         </is>
       </c>
     </row>

</xml_diff>